<commit_message>
Pregenerisani proracuni, Prilog III i DWG izvozi
</commit_message>
<xml_diff>
--- a/rfp-hybrid-solar-td/TD-OUTPUT/3.1 PRILOG II TD - Obrazac za cijenu ponude LOT 1 - Sjednica i Hamzici.xlsx
+++ b/rfp-hybrid-solar-td/TD-OUTPUT/3.1 PRILOG II TD - Obrazac za cijenu ponude LOT 1 - Sjednica i Hamzici.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="LOT 1 Sjednica" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="LOT 1 Hamzići" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="REKAPITULACIJA LOT 1" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LOT 1 Sjednica" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LOT 1 Hamzići" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REKAPITULACIJA LOT 1" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'LOT 1 Sjednica'!$8:$9</definedName>

</xml_diff>

<commit_message>
Silueta stuba H-06 centrirana, formalne i manje napomene, trake FN u nivou ploče na Hamzićima
- extract_tower.py: osa stuba je sredina cijele siluete; kod Hamzića je stub ispadao
  pomaknut za pola baze udesno (H-06). tower_profile.json Hamzića ponovo izvučen.
- Napomene na svim listovima: tekst 1,7 mm (naslov 2,2 mm), jednopolne šeme 1,5 mm;
  formulacije u punim rečenicama, bez skraćenica i verzala.
- Hamzići: vrh temeljnih traka u nivou ploče, 0,20 m iznad terena (Naručilac
  05.10.2026). Kote polja od ploče (+0,50 / +2,93), nadvišenje ograde 1,13 m.
  Traka ista (900 mm, 9,36 m³), rov 750 mm: iskop i odvoz 7,80 m³, obrada 20,3 m².
  H-03 i H-06 pregenerisani; Prilog I, Prilog II, proračuni i provjere usklađeni.
</commit_message>
<xml_diff>
--- a/rfp-hybrid-solar-td/TD-OUTPUT/3.1 PRILOG II TD - Obrazac za cijenu ponude LOT 1 - Sjednica i Hamzici.xlsx
+++ b/rfp-hybrid-solar-td/TD-OUTPUT/3.1 PRILOG II TD - Obrazac za cijenu ponude LOT 1 - Sjednica i Hamzici.xlsx
@@ -1916,8 +1916,8 @@
           <t>Isporuka i montaža nosive metalne konstrukcije (ground mount support) za prihvat fotonaponskih panela:
  - 4 odvojena nosača u jednom nizu, svaki za 3 fotonaponska modula (3 reda × 1 kolona, položeno); razmak između nosača 400 mm, dužina niza 10 312 mm
  - nagib fiksno 45°, orijentacija JUGOZAPAD (azimut 225°), niz paralelan sa jugozapadnom ogradom
- - gabariti po nosaču: širina polja 2278 mm (poprečna greda 2891 mm, bočni prepust 306,5 mm), dužina polja po nagibu 3442 mm, horizontalna projekcija 2434 mm pri nagibu 45°; donja ivica panela na +0,50 m, gornja ivica na +2,93 m od nivoa terena
- - smještaj (43,288012° N, 17,624794° E, 493 m n.v.): nosači se temelje IZVAN ograđenog platoa, jugozapadno od ploče i ograde, u pojasu dubine 3300 mm i dužine 12,50 m (JZ strana), unutar zakupa k.č. 109/1 K.O. Hamzići (12,00 × 12,50 m); trake 350 mm od granice zakupa i od ploče; gornja (sjeveroistočna) ivica panela je 0,93 m iznad vrha ograde — ograda je h=1,80 m iznad ploče, odnosno 2,00 m iznad vanjskog terena, koji je uz ploču na −0,20 m (ovjereni 04_Ograda)
+ - gabariti po nosaču: širina polja 2278 mm (poprečna greda 2891 mm, bočni prepust 306,5 mm), dužina polja po nagibu 3442 mm, horizontalna projekcija 2434 mm pri nagibu 45°; donja ivica panela na +0,50 m, gornja ivica na +2,93 m od gornje ivice ploče, u čijem je nivou vrh temeljnih traka
+ - smještaj (43,288012° N, 17,624794° E, 493 m n.v.): nosači se temelje IZVAN ograđenog platoa, jugozapadno od ploče i ograde, u pojasu dubine 3300 mm i dužine 12,50 m (JZ strana), unutar zakupa k.č. 109/1 K.O. Hamzići (12,00 × 12,50 m); trake 350 mm od granice zakupa i od ploče; vrh temeljnih traka je u nivou gornje ivice ploče, 0,20 m iznad vanjskog terena (teren uz ploču je na −0,20 m, ovjereni 04_Ograda); gornja (sjeveroistočna) ivica panela je 1,13 m iznad vrha ograde h=1,80 m od ploče
  - materijal, antikorozivna zaštita, zavarivanje i spojni pribor prema Prilogu I, Tačka 3.3
  - uključeno ožičenje i povezivanje panela do PVDB distribucije preko po-string DC odvodnika prenapona (v. crtež H-05): 12 modula se povezuje u DVA STRINGA po 6 modula (string 1 — nosači PV-1 i PV-2; string 2 — nosači PV-3 i PV-4), po jedan string na svaku od dvije rute PVDB ormara
  - UZ PONUDU: Ponuđač je obavezan da uz ponudu dostavi tehničko rješenje konstrukcije za prihvat fotonaponskih panela za predmetnu lokaciju, sa obaveznim statičkim proračunom (Tačka 1.3) i specifikacijom materijala. Tehničko rješenje mora biti pregledano i odobreno prije početka izvođenja radova</t>
@@ -2116,7 +2116,7 @@
       </c>
       <c r="B21" s="129" t="inlineStr">
         <is>
-          <t>Iskop zemlje/stijene IV-V kategorije za temeljne trake nosača, do donje ivice podložnog betona. Rov širine 500 mm, dubine 950 mm, dužine 2600 mm. 4 nosača × 2 trake × 1,235 m3. Rov se u stijeni siječe jednom širinom po cijeloj dubini; traka se betonira do zida rova, pa zatrpavanja nema.</t>
+          <t>Iskop zemlje/stijene IV-V kategorije za temeljne trake nosača, do donje ivice podložnog betona. Rov širine 500 mm, dubine 750 mm od vanjskog terena, dužine 2600 mm (vrh trake je 0,20 m iznad terena, u nivou ploče). 4 nosača × 2 trake × 0,975 m3. Rov se u stijeni siječe jednom širinom po cijeloj dubini; traka se betonira do zida rova, pa zatrpavanja nema.</t>
         </is>
       </c>
       <c r="C21" s="130" t="inlineStr">
@@ -2125,7 +2125,7 @@
         </is>
       </c>
       <c r="D21" s="130" t="n">
-        <v>9.880000000000001</v>
+        <v>7.8</v>
       </c>
       <c r="E21" s="131" t="n"/>
       <c r="F21" s="131">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="B22" s="129" t="inlineStr">
         <is>
-          <t>Odvoz i zbrinjavanje viška materijala od iskopa do deponije udaljene do 20 km. Traka i podložni beton ispunjavaju rov u cijelosti, pa se odvozi sav iskopani materijal. 4 nosača × 2 trake × 1,235 m3</t>
+          <t>Odvoz i zbrinjavanje viška materijala od iskopa do deponije udaljene do 20 km. Traka i podložni beton ispunjavaju rov u cijelosti, pa se odvozi sav iskopani materijal. 4 nosača × 2 trake × 0,975 m3</t>
         </is>
       </c>
       <c r="C22" s="130" t="inlineStr">
@@ -2150,7 +2150,7 @@
         </is>
       </c>
       <c r="D22" s="130" t="n">
-        <v>9.880000000000001</v>
+        <v>7.8</v>
       </c>
       <c r="E22" s="131" t="n"/>
       <c r="F22" s="131">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="B24" s="129" t="inlineStr">
         <is>
-          <t>Nabavka materijala, transport i betoniranje DVIJE temeljne trake po nosaču, betonom C30/37 klase izloženosti XC4 + XF3 prema BAS EN 206 (aerant 4–6 %, Dmax 16, konzistencija S3), uz upotrebu oplate i njegovanje betona. Armatura B500B, zaštitni sloj ≥50 mm, prema ovjerenom statičkom proračunu iz Tačke 1.3. Obračun po m³ ugrađenog betona. Traka 500 × 2600 mm, jedinstvene širine po cijeloj dubini (bez proširenja u dnu), PUNE dubine 900 mm = 1,170 m³ po traci. 4 nosača × 2 trake × 1,170 m³
+          <t>Nabavka materijala, transport i betoniranje DVIJE temeljne trake po nosaču, betonom C30/37 klase izloženosti XC4 + XF3 prema BAS EN 206 (aerant 4–6 %, Dmax 16, konzistencija S3), uz upotrebu oplate i njegovanje betona. Armatura B500B, zaštitni sloj ≥50 mm, prema ovjerenom statičkom proračunu iz Tačke 1.3. Obračun po m³ ugrađenog betona. Traka 500 × 2600 mm, jedinstvene širine po cijeloj dubini (bez proširenja u dnu), PUNE dubine 900 mm = 1,170 m³ po traci; vrh trake je u nivou gornje ivice ploče, 0,20 m iznad vanjskog terena, pa se gornjih 200 mm betonira u oplati. 4 nosača × 2 trake × 1,170 m³
 BETON I ARMATURA: beton klase C30/37, klase izloženosti XC4 + XF3 prema BAS EN 206, sa aerantom 4–6 %, Dmax 16, konzistencija S3; podložni beton C12/15 d=50 mm; armatura B500B, zaštitni sloj ≥50 mm. Klasa XF3: ista specifikacija kao na lokaciji Sjednica, radi jednog opisa za obje lokacije. Temeljna spojnica mora biti ispod dubine smrzavanja za lokalitet, koju Ponuđač navodi u ponudi. Dubina 900 mm je tenderska osnova i mjerodavna je za ponudu; konačnu dubinu i armaturu potvrđuje ovjereni statički proračun iz Tačke 1.3. Traka se betonira punom dubinom rova i do zida rova — vlastita težina trake je dio dokaza sigurnosti na podizanje i prevrtanje. Temelj širi u dnu nego u vrhu tražio bi potkopavanje i u stijeni nije izvodiv, pa je presjek jedinstven.</t>
         </is>
       </c>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="B25" s="129" t="inlineStr">
         <is>
-          <t>Obrada vidljivih strana i gornje površine temeljnih traka cementnim malterom u nagibu 1,0 %, zaglađeno do crnog sjaja. 0,50 × 2,60 × 8 traka = 10,4 m².</t>
+          <t>Obrada vidljivih strana i gornje površine temeljnih traka cementnim malterom u nagibu 1,0 %, zaglađeno do crnog sjaja. Gornja površina 0,50 × 2,60 × 8 traka = 10,4 m² i bočne strane iznad terena 2 × (2,60 + 0,50) × 0,20 × 8 traka = 9,9 m², ukupno 20,3 m².</t>
         </is>
       </c>
       <c r="C25" s="130" t="inlineStr">
@@ -2226,7 +2226,7 @@
         </is>
       </c>
       <c r="D25" s="130" t="n">
-        <v>10.4</v>
+        <v>20.3</v>
       </c>
       <c r="E25" s="131" t="n"/>
       <c r="F25" s="131">

</xml_diff>

<commit_message>
Kratke formalne napomene; Prilog II ostaje kako je izdat
- Napomene na svim listovima skraćene: jedna rečenica po tački, formalno.
- Prilog II se ne mijenja (Naručilac 05.10.2026): joint_boq.py, check_boq_recalc.py i
  oba obrasca vraćeni na main; količine iskopa, odvoza i obrade ostaju 9,88 / 9,88 /
  10,4. Prilog I, proračuni i design.json ne navode nove količine; ostaje samo kota
  traka u nivou ploče i nadvišenje ograde 1,13 m.
- rules_joint: 0,93 m u stavci 1.1 izdatog Priloga II nije greška.
</commit_message>
<xml_diff>
--- a/rfp-hybrid-solar-td/TD-OUTPUT/3.1 PRILOG II TD - Obrazac za cijenu ponude LOT 1 - Sjednica i Hamzici.xlsx
+++ b/rfp-hybrid-solar-td/TD-OUTPUT/3.1 PRILOG II TD - Obrazac za cijenu ponude LOT 1 - Sjednica i Hamzici.xlsx
@@ -1916,8 +1916,8 @@
           <t>Isporuka i montaža nosive metalne konstrukcije (ground mount support) za prihvat fotonaponskih panela:
  - 4 odvojena nosača u jednom nizu, svaki za 3 fotonaponska modula (3 reda × 1 kolona, položeno); razmak između nosača 400 mm, dužina niza 10 312 mm
  - nagib fiksno 45°, orijentacija JUGOZAPAD (azimut 225°), niz paralelan sa jugozapadnom ogradom
- - gabariti po nosaču: širina polja 2278 mm (poprečna greda 2891 mm, bočni prepust 306,5 mm), dužina polja po nagibu 3442 mm, horizontalna projekcija 2434 mm pri nagibu 45°; donja ivica panela na +0,50 m, gornja ivica na +2,93 m od gornje ivice ploče, u čijem je nivou vrh temeljnih traka
- - smještaj (43,288012° N, 17,624794° E, 493 m n.v.): nosači se temelje IZVAN ograđenog platoa, jugozapadno od ploče i ograde, u pojasu dubine 3300 mm i dužine 12,50 m (JZ strana), unutar zakupa k.č. 109/1 K.O. Hamzići (12,00 × 12,50 m); trake 350 mm od granice zakupa i od ploče; vrh temeljnih traka je u nivou gornje ivice ploče, 0,20 m iznad vanjskog terena (teren uz ploču je na −0,20 m, ovjereni 04_Ograda); gornja (sjeveroistočna) ivica panela je 1,13 m iznad vrha ograde h=1,80 m od ploče
+ - gabariti po nosaču: širina polja 2278 mm (poprečna greda 2891 mm, bočni prepust 306,5 mm), dužina polja po nagibu 3442 mm, horizontalna projekcija 2434 mm pri nagibu 45°; donja ivica panela na +0,50 m, gornja ivica na +2,93 m od nivoa terena
+ - smještaj (43,288012° N, 17,624794° E, 493 m n.v.): nosači se temelje IZVAN ograđenog platoa, jugozapadno od ploče i ograde, u pojasu dubine 3300 mm i dužine 12,50 m (JZ strana), unutar zakupa k.č. 109/1 K.O. Hamzići (12,00 × 12,50 m); trake 350 mm od granice zakupa i od ploče; gornja (sjeveroistočna) ivica panela je 0,93 m iznad vrha ograde — ograda je h=1,80 m iznad ploče, odnosno 2,00 m iznad vanjskog terena, koji je uz ploču na −0,20 m (ovjereni 04_Ograda)
  - materijal, antikorozivna zaštita, zavarivanje i spojni pribor prema Prilogu I, Tačka 3.3
  - uključeno ožičenje i povezivanje panela do PVDB distribucije preko po-string DC odvodnika prenapona (v. crtež H-05): 12 modula se povezuje u DVA STRINGA po 6 modula (string 1 — nosači PV-1 i PV-2; string 2 — nosači PV-3 i PV-4), po jedan string na svaku od dvije rute PVDB ormara
  - UZ PONUDU: Ponuđač je obavezan da uz ponudu dostavi tehničko rješenje konstrukcije za prihvat fotonaponskih panela za predmetnu lokaciju, sa obaveznim statičkim proračunom (Tačka 1.3) i specifikacijom materijala. Tehničko rješenje mora biti pregledano i odobreno prije početka izvođenja radova</t>
@@ -2116,7 +2116,7 @@
       </c>
       <c r="B21" s="129" t="inlineStr">
         <is>
-          <t>Iskop zemlje/stijene IV-V kategorije za temeljne trake nosača, do donje ivice podložnog betona. Rov širine 500 mm, dubine 750 mm od vanjskog terena, dužine 2600 mm (vrh trake je 0,20 m iznad terena, u nivou ploče). 4 nosača × 2 trake × 0,975 m3. Rov se u stijeni siječe jednom širinom po cijeloj dubini; traka se betonira do zida rova, pa zatrpavanja nema.</t>
+          <t>Iskop zemlje/stijene IV-V kategorije za temeljne trake nosača, do donje ivice podložnog betona. Rov širine 500 mm, dubine 950 mm, dužine 2600 mm. 4 nosača × 2 trake × 1,235 m3. Rov se u stijeni siječe jednom širinom po cijeloj dubini; traka se betonira do zida rova, pa zatrpavanja nema.</t>
         </is>
       </c>
       <c r="C21" s="130" t="inlineStr">
@@ -2125,7 +2125,7 @@
         </is>
       </c>
       <c r="D21" s="130" t="n">
-        <v>7.8</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="E21" s="131" t="n"/>
       <c r="F21" s="131">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="B22" s="129" t="inlineStr">
         <is>
-          <t>Odvoz i zbrinjavanje viška materijala od iskopa do deponije udaljene do 20 km. Traka i podložni beton ispunjavaju rov u cijelosti, pa se odvozi sav iskopani materijal. 4 nosača × 2 trake × 0,975 m3</t>
+          <t>Odvoz i zbrinjavanje viška materijala od iskopa do deponije udaljene do 20 km. Traka i podložni beton ispunjavaju rov u cijelosti, pa se odvozi sav iskopani materijal. 4 nosača × 2 trake × 1,235 m3</t>
         </is>
       </c>
       <c r="C22" s="130" t="inlineStr">
@@ -2150,7 +2150,7 @@
         </is>
       </c>
       <c r="D22" s="130" t="n">
-        <v>7.8</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="E22" s="131" t="n"/>
       <c r="F22" s="131">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="B24" s="129" t="inlineStr">
         <is>
-          <t>Nabavka materijala, transport i betoniranje DVIJE temeljne trake po nosaču, betonom C30/37 klase izloženosti XC4 + XF3 prema BAS EN 206 (aerant 4–6 %, Dmax 16, konzistencija S3), uz upotrebu oplate i njegovanje betona. Armatura B500B, zaštitni sloj ≥50 mm, prema ovjerenom statičkom proračunu iz Tačke 1.3. Obračun po m³ ugrađenog betona. Traka 500 × 2600 mm, jedinstvene širine po cijeloj dubini (bez proširenja u dnu), PUNE dubine 900 mm = 1,170 m³ po traci; vrh trake je u nivou gornje ivice ploče, 0,20 m iznad vanjskog terena, pa se gornjih 200 mm betonira u oplati. 4 nosača × 2 trake × 1,170 m³
+          <t>Nabavka materijala, transport i betoniranje DVIJE temeljne trake po nosaču, betonom C30/37 klase izloženosti XC4 + XF3 prema BAS EN 206 (aerant 4–6 %, Dmax 16, konzistencija S3), uz upotrebu oplate i njegovanje betona. Armatura B500B, zaštitni sloj ≥50 mm, prema ovjerenom statičkom proračunu iz Tačke 1.3. Obračun po m³ ugrađenog betona. Traka 500 × 2600 mm, jedinstvene širine po cijeloj dubini (bez proširenja u dnu), PUNE dubine 900 mm = 1,170 m³ po traci. 4 nosača × 2 trake × 1,170 m³
 BETON I ARMATURA: beton klase C30/37, klase izloženosti XC4 + XF3 prema BAS EN 206, sa aerantom 4–6 %, Dmax 16, konzistencija S3; podložni beton C12/15 d=50 mm; armatura B500B, zaštitni sloj ≥50 mm. Klasa XF3: ista specifikacija kao na lokaciji Sjednica, radi jednog opisa za obje lokacije. Temeljna spojnica mora biti ispod dubine smrzavanja za lokalitet, koju Ponuđač navodi u ponudi. Dubina 900 mm je tenderska osnova i mjerodavna je za ponudu; konačnu dubinu i armaturu potvrđuje ovjereni statički proračun iz Tačke 1.3. Traka se betonira punom dubinom rova i do zida rova — vlastita težina trake je dio dokaza sigurnosti na podizanje i prevrtanje. Temelj širi u dnu nego u vrhu tražio bi potkopavanje i u stijeni nije izvodiv, pa je presjek jedinstven.</t>
         </is>
       </c>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="B25" s="129" t="inlineStr">
         <is>
-          <t>Obrada vidljivih strana i gornje površine temeljnih traka cementnim malterom u nagibu 1,0 %, zaglađeno do crnog sjaja. Gornja površina 0,50 × 2,60 × 8 traka = 10,4 m² i bočne strane iznad terena 2 × (2,60 + 0,50) × 0,20 × 8 traka = 9,9 m², ukupno 20,3 m².</t>
+          <t>Obrada vidljivih strana i gornje površine temeljnih traka cementnim malterom u nagibu 1,0 %, zaglađeno do crnog sjaja. 0,50 × 2,60 × 8 traka = 10,4 m².</t>
         </is>
       </c>
       <c r="C25" s="130" t="inlineStr">
@@ -2226,7 +2226,7 @@
         </is>
       </c>
       <c r="D25" s="130" t="n">
-        <v>20.3</v>
+        <v>10.4</v>
       </c>
       <c r="E25" s="131" t="n"/>
       <c r="F25" s="131">

</xml_diff>